<commit_message>
LichPhylactery 1.75.0 - 1.89.0
- 1.75.0 非战斗经验 / 磨砺; 1.76.0 初始属性购点; 1.77.0 装备贴图重画
- 1.78.0 野蛮人/游侠/游荡者; 1.79.0 15 个新强力特性; 1.80.0 野外怪物
- 1.81.0 子职业、职业生命骰、职业平衡修复; 1.82.0 邪术师与 NPC 职业、已知问题修复
- 1.83.0 探索公告板奖励; 1.84.0 职业能力自动施放; 1.85.0 附魔强化 +1..+10
- 1.86.0 Character Editor 联动; 1.87.0 职业等级 15 级终极特性
- 1.88.0 职业专属专长; 1.89.0 职业界面（部位生命/职业能力前后对比）
- 属性页、研究速度修复、各项热修复

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ArtSource/DND特性与冲突.xlsx
+++ b/ArtSource/DND特性与冲突.xlsx
@@ -14,9 +14,9 @@
     <sheet name="获得规则" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'特性一览'!$A$1:$I$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'稀有度'!$A$1:$E$135</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'冲突对照'!$A$1:$E$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'特性一览'!$A$1:$I$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'稀有度'!$A$1:$E$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'冲突对照'!$A$1:$E$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'互斥组'!$A$1:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'获得规则'!$A$1:$D$11</definedName>
   </definedNames>
@@ -543,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 2 个）</t>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 6 个）</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 2 个）</t>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 6 个）</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 2 个）</t>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 6 个）</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -4004,8 +4004,653 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>巧匠之手</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>LP_Artisan</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的手好像天生就知道该怎么用工具。\n\n- 全局工作速度 +10%\n- 传奇属性“工作”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>诅咒 · 稀有</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>厄运缠身</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>LP_Doomed</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 6 个）</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">一个女巫在临死前诅咒了{PAWN_nameDef}。厄运一直跟着{PAWN_objective}，有时也会扑向别人。\n\n- 近战闪避 +15\n- 被敌人打中时 15% 的几率「厄运转嫁」：攻击者也受到这次伤害的一半\n- 代价：平均每 8 天一次厄运降临——身上一件衣甲耐久 -30%，心情 -5「厄运缠身」（2 </t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>远瞳</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>LP_EagleEyed</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}能看清别人只看得到一个黑点的东西。\n\n- 射击精度 +6\n- 瞄准时间 ×0.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>处刑者</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>LP_Executioner</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}看得出谁已经撑不住了，下手从不留情。\n\n- 对倒地、或者总体健康低于 30% 的敌人伤害 +50%\n- 亲手击杀敌人后 1 小时内近战与射击命中 +10%「乘胜追击」</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>疾风之足</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>LP_Fleetfoot</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}跑起来像一阵风。\n\n- 移动速度 +0.4\n- 近战闪避 +10</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>荒野之躯</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>LP_Hardy</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}在荒野里摸爬滚打长大，什么苦都吃过。\n\n- 免疫获得速度 ×1.2\n- 伤口愈合速度 ×1.3\n- 毒素抗性 +25%\n- 舒适温度范围两头各放宽 10°C</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="inlineStr">
+        <is>
+          <t>诅咒 · 史诗</t>
+        </is>
+      </c>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>狱火烙印</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>LP_Hellbrand</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 6 个）</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的胸口有一个九狱魔鬼留下的烙印，到现在还是烫的。\n\n- 武器命中额外造成 4 点火焰伤害\n- 受到的火焰类伤害 -75%\n- 舒适温度上限 +40°C\n- 代价：受到的寒冷类伤害 +50%；精神崩溃阈值 +5%；平均每 12 天一次魔鬼来索债，心情 -8「狱火索债」（3 天）</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="inlineStr">
+        <is>
+          <t>诅咒 · 稀有</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>空心之人</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>LP_Hollow</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 6 个）</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的一半灵魂被什么东西吃掉了，剩下的那一半很平静——平静得吓人。\n\n- 精神崩溃阈值 -15%\n- 疼痛休克阈值 +20%\n- 心智抗性 +50%\n- 代价：社交影响 ×0.5、技能学习速度 ×0.8、心灵敏感度 -30%、外貌 -1（别人看着发怵）</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>钢铁意志</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>LP_IronWill</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的意志像铁一样硬，什么都压不垮。\n\n- 精神崩溃阈值 -8%\n- 心智抗性 +30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>万夫莫敌</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>LP_Juggernaut</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}挨刀子就像挨了一拳。\n\n- 受到的伤害 ×0.85\n- 疼痛休克阈值 +15%\n- 传奇属性“血量”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B89" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>神童</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>LP_Prodigy</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}学什么都比别人快一大截。\n\n- 技能学习速度 ×1.5\n- 传奇属性“学习”“工作”每点收益 ×1.5（与种族亲和取较大，不相乘）\n- 智力上限 +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>银舌</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>LP_Silvertongue</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}一开口，石头都能被说动。\n\n- 谈判能力 ×1.3、社交影响 ×1.3\n- 魅力上限 +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B91" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>魔裔之血</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>LP_Spellblood</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>法术抗体</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的祖上和某种魔法生物通过婚，魔网在{PAWN_possessive}血里流淌。\n\n- 心灵敏感度 +25%\n- 心灵熵恢复速度 ×1.3\n- 传奇属性“心灵”每点收益 ×2（与种族亲和取较大，不相乘）\n- 不会和法术抗体同时出现</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>百折不挠</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>LP_Unyielding</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}好几次都该死了，可每次都又爬了起来。\n\n- 致命伤改为倒地幸存，伤口止血（冷却 10 天，处决和手术不算）\n- 和命运之恩、命运未尽不会同一次触发：它们先判\n- 疼痛休克阈值 +10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>HeroTraits_More.xml</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="inlineStr">
+        <is>
+          <t>诅咒 · 史诗</t>
+        </is>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>吸血鬼之咒</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>LP_Vampirism</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）（同组 6 个）</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}被吸血鬼咬过，没死，可也不再完全是活人了。\n\n- 近战伤害 ×1.3，移动速度 +0.3\n- 伤口愈合速度 ×2\n- 近战命中时吸血，回复 2 点伤势\n- 代价：白天待在没有屋顶的地方会「日光灼身」——移动 -15%、意识 -10%，每小时受到 1 点烧伤；进屋或天黑就消退</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I78"/>
+  <autoFilter ref="A1:I93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4016,7 +4661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5161,218 +5806,218 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>神童</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>LP_Prodigy</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}学什么都比别人快一大截。\n\n- 技能学习速度 ×1.5\n- 传奇属性“学习”“工作”每点收益 ×1.5（与种族亲和取较大，不相乘）\n- 智力上限 +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>百折不挠</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>LP_Unyielding</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}好几次都该死了，可每次都又爬了起来。\n\n- 致命伤改为倒地幸存，伤口止血（冷却 10 天，处决和手术不算）\n- 和命运之恩、命运未尽不会同一次触发：它们先判\n- 疼痛休克阈值 +10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>万夫莫敌</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>LP_Juggernaut</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}挨刀子就像挨了一拳。\n\n- 受到的伤害 ×0.85\n- 疼痛休克阈值 +15%\n- 传奇属性“血量”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>魔裔之血</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>LP_Spellblood</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的祖上和某种魔法生物通过婚，魔网在{PAWN_possessive}血里流淌。\n\n- 心灵敏感度 +25%\n- 心灵熵恢复速度 ×1.3\n- 传奇属性“心灵”每点收益 ×2（与种族亲和取较大，不相乘）\n</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>处刑者</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>LP_Executioner</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}看得出谁已经撑不住了，下手从不留情。\n\n- 对倒地、或者总体健康低于 30% 的敌人伤害 +50%\n- 亲手击杀敌人后 1 小时内近战与射击命中 +10%「乘胜追击」</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>史诗（诅咒）</t>
+        </is>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>吸血鬼之咒</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>LP_Vampirism</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}被吸血鬼咬过，没死，可也不再完全是活人了。\n\n- 近战伤害 ×1.3，移动速度 +0.3\n- 伤口愈合速度 ×2\n- 近战命中时吸血，回复 2 点伤势\n- 代价：白天待在没有屋顶的地方会「日光灼身」——</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>史诗（诅咒）</t>
+        </is>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>狱火烙印</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>LP_Hellbrand</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的胸口有一个九狱魔鬼留下的烙印，到现在还是烫的。\n\n- 武器命中额外造成 4 点火焰伤害\n- 受到的火焰类伤害 -75%\n- 舒适温度上限 +40°C\n- 代价：受到的寒冷类伤害 +50%；精神崩溃阈值</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>稀有（事迹）</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>弑神者</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>LP_Godslayer</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>传说事迹</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>[PAWN_nameDef]亲手击败过神明附体的首领：对神力灌注者、神明附体者和半神造成的伤害×1.3；神明附体首领的神技打在[PAWN_objective]身上只有七成效果。</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>巨力</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>LP_CG_Mighty</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>武艺天赋</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}天生神力，抡起战锤像抡起柴刀。\n\n入门：力量 +2（上限 +2）；负重 +25%</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>迅捷</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>LP_CG_Swift</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>武艺天赋</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}的脚步轻得像风，没人追得上。\n\n入门：敏捷 +2（上限 +2）；移动速度 +0.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>坚韧之体</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>LP_CG_Stalwart</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>武艺天赋</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}的骨头比铁还硬，挨了刀也只是皱皱眉。\n\n入门：体质 +2（上限 +2）；受到的伤害 -10%（最多 -25%）</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>博闻强识</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>LP_CG_Brilliant</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>武艺天赋</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}过目不忘，任何典籍读一遍就能复述。\n\n入门：智力 +2（上限 +2）；研究速度 +15%</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>鹰眼</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>LP_CG_Eagle</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>武艺天赋</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}能在百步之外看清敌人的眼神。\n\n入门：感知 +2（上限 +2）；远程瞄准时间 -20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>王者气度</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>LP_CG_Commanding</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>武艺天赋</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}一开口，所有人都会安静下来听。\n\n入门：魅力 +2（上限 +2）；社交影响 +20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>连斩</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>LP_CG_Flurry</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>武艺天赋</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}的刀快得只剩残影。\n\n入门：近战冷却 -20%；近战命中后成功率 15% 立刻追加一击</t>
         </is>
       </c>
     </row>
@@ -5384,12 +6029,12 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>狂暴之血</t>
+          <t>巨力</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>LP_CG_Rage</t>
+          <t>LP_CG_Mighty</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -5399,7 +6044,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>越是伤重，{PAWN_nameDef}越是凶猛。\n\n入门：健康低于 60% 时近战伤害 +30%、近战冷却 -15%、疼痛 ×0.5</t>
+          <t>{PAWN_nameDef}天生神力，抡起战锤像抡起柴刀。\n\n入门：力量 +2（上限 +2）；负重 +25%</t>
         </is>
       </c>
     </row>
@@ -5411,12 +6056,12 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>神射</t>
+          <t>迅捷</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>LP_CG_Deadeye</t>
+          <t>LP_CG_Swift</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -5426,7 +6071,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}射出的箭和子弹好像长了眼睛。\n\n入门：远程命中 +12%；远程伤害 +15%</t>
+          <t>{PAWN_nameDef}的脚步轻得像风，没人追得上。\n\n入门：敏捷 +2（上限 +2）；移动速度 +0.4</t>
         </is>
       </c>
     </row>
@@ -5438,12 +6083,12 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>致命一击</t>
+          <t>坚韧之体</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>LP_CG_Lethal</t>
+          <t>LP_CG_Stalwart</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -5453,7 +6098,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}总能找到对手的要害。\n\n入门：任何攻击成功率 10% 暴击，伤害 ×2；护甲穿透 +10%</t>
+          <t>{PAWN_nameDef}的骨头比铁还硬，挨了刀也只是皱皱眉。\n\n入门：体质 +2（上限 +2）；受到的伤害 -10%（最多 -25%）</t>
         </is>
       </c>
     </row>
@@ -5465,12 +6110,12 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>铁壁</t>
+          <t>博闻强识</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>LP_CG_Bulwark</t>
+          <t>LP_CG_Brilliant</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -5480,7 +6125,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}站稳了就像一堵墙。\n\n入门：利器 / 钝器护甲 +15%（绝对值，最多 +30%）；不会踉跄</t>
+          <t>{PAWN_nameDef}过目不忘，任何典籍读一遍就能复述。\n\n入门：智力 +2（上限 +2）；研究速度 +15%</t>
         </is>
       </c>
     </row>
@@ -5492,12 +6137,12 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>再生之体</t>
+          <t>鹰眼</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>LP_CG_Regen</t>
+          <t>LP_CG_Eagle</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -5507,7 +6152,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}的伤口愈合得惊人地快，断肢也能慢慢长回来。\n\n入门：伤口愈合 ×2.5；每 15 天长回一个缺失的非要害部位</t>
+          <t>{PAWN_nameDef}能在百步之外看清敌人的眼神。\n\n入门：感知 +2（上限 +2）；远程瞄准时间 -20%</t>
         </is>
       </c>
     </row>
@@ -5519,12 +6164,12 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>法力奔涌</t>
+          <t>王者气度</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>LP_CG_Arcane</t>
+          <t>LP_CG_Commanding</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -5534,34 +6179,34 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>魔力在{PAWN_nameDef}的血管里奔流。\n\n入门：法杖 / 灵能 / 神术伤害 +25%；装了 VPE 时心灵熵上限 +20，否则心灵敏感度 +15%</t>
+          <t>{PAWN_nameDef}一开口，所有人都会安静下来听。\n\n入门：魅力 +2（上限 +2）；社交影响 +20%</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="15" t="inlineStr">
-        <is>
-          <t>稀有（诅咒）</t>
-        </is>
-      </c>
-      <c r="B57" s="16" t="inlineStr">
-        <is>
-          <t>远域之触</t>
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>连斩</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>LP_FarRealmTouched</t>
+          <t>LP_CG_Flurry</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>诅咒之力</t>
+          <t>武艺天赋</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>群星之外的东西碰过{PAWN_nameDef}的心智，留下了一道缝。\n\n- 心灵敏感度 +40%，心灵熵上限 +20\n- 能力「心灵冲击」：前方 5 格锥形内的敌人眩晕 2 秒并受到 15 点灵能伤害，每天 3 次\n- 地图上出现敌</t>
+          <t>{PAWN_nameDef}的刀快得只剩残影。\n\n入门：近战冷却 -20%；近战命中后成功率 15% 立刻追加一击</t>
         </is>
       </c>
     </row>
@@ -5573,22 +6218,22 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>天赋·力量</t>
+          <t>狂暴之血</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>LP_GiftedScore(1)</t>
+          <t>LP_CG_Rage</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>强力特性</t>
+          <t>武艺天赋</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}天生力气大。\n\n- 力量算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>越是伤重，{PAWN_nameDef}越是凶猛。\n\n入门：健康低于 60% 时近战伤害 +30%、近战冷却 -15%、疼痛 ×0.5</t>
         </is>
       </c>
     </row>
@@ -5600,22 +6245,22 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>天赋·敏捷</t>
+          <t>神射</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>LP_GiftedScore(2)</t>
+          <t>LP_CG_Deadeye</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>强力特性</t>
+          <t>武艺天赋</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}天生手脚灵活。\n\n- 敏捷算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>{PAWN_nameDef}射出的箭和子弹好像长了眼睛。\n\n入门：远程命中 +12%；远程伤害 +15%</t>
         </is>
       </c>
     </row>
@@ -5627,22 +6272,22 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>天赋·体质</t>
+          <t>致命一击</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>LP_GiftedScore(3)</t>
+          <t>LP_CG_Lethal</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>强力特性</t>
+          <t>武艺天赋</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}天生结实。\n\n- 体质算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>{PAWN_nameDef}总能找到对手的要害。\n\n入门：任何攻击成功率 10% 暴击，伤害 ×2；护甲穿透 +10%</t>
         </is>
       </c>
     </row>
@@ -5654,22 +6299,22 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>天赋·智力</t>
+          <t>铁壁</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>LP_GiftedScore(4)</t>
+          <t>LP_CG_Bulwark</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>强力特性</t>
+          <t>武艺天赋</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}天生聪明。\n\n- 智力算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>{PAWN_nameDef}站稳了就像一堵墙。\n\n入门：利器 / 钝器护甲 +15%（绝对值，最多 +30%）；不会踉跄</t>
         </is>
       </c>
     </row>
@@ -5681,22 +6326,22 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>天赋·感知</t>
+          <t>再生之体</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>LP_GiftedScore(5)</t>
+          <t>LP_CG_Regen</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>强力特性</t>
+          <t>武艺天赋</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}天生敏锐。\n\n- 感知算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>{PAWN_nameDef}的伤口愈合得惊人地快，断肢也能慢慢长回来。\n\n入门：伤口愈合 ×2.5；每 15 天长回一个缺失的非要害部位</t>
         </is>
       </c>
     </row>
@@ -5708,49 +6353,49 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>天赋·魅力</t>
+          <t>法力奔涌</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>LP_GiftedScore(6)</t>
+          <t>LP_CG_Arcane</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>强力特性</t>
+          <t>武艺天赋</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}天生讨人喜欢。\n\n- 魅力算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>魔力在{PAWN_nameDef}的血管里奔流。\n\n入门：法杖 / 灵能 / 神术伤害 +25%；装了 VPE 时心灵熵上限 +20，否则心灵敏感度 +15%</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>稀有</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>金刚之躯</t>
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>稀有（诅咒）</t>
+        </is>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>远域之触</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>LP_Hardened</t>
+          <t>LP_FarRealmTouched</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>强力特性</t>
+          <t>诅咒之力</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}的身子骨像铁打的。\n\n- 传奇属性“血量”“承受”“回复”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>群星之外的东西碰过{PAWN_nameDef}的心智，留下了一道缝。\n\n- 心灵敏感度 +40%，心灵熵上限 +20\n- 能力「心灵冲击」：前方 5 格锥形内的敌人眩晕 2 秒并受到 15 点灵能伤害，每天 3 次\n- 地图上出现敌</t>
         </is>
       </c>
     </row>
@@ -5762,12 +6407,12 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>锋芒</t>
+          <t>天赋·力量</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>LP_Edge</t>
+          <t>LP_GiftedScore(1)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -5777,7 +6422,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}生来就是打仗的料。\n\n- 传奇属性“近战”“远程”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
+          <t>{PAWN_nameDef}天生力气大。\n\n- 力量算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5789,12 +6434,12 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>灵光</t>
+          <t>天赋·敏捷</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>LP_Insight</t>
+          <t>LP_GiftedScore(2)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -5804,7 +6449,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}的脑子里时常闪过别人想不到的东西。\n\n- 传奇属性“心灵”“学习”每点收益 ×1.5（与种族亲和取较大，不相乘）\n- 智力、感知中较高的一项上限 +2</t>
+          <t>{PAWN_nameDef}天生手脚灵活。\n\n- 敏捷算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5816,12 +6461,12 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>传奇之胚</t>
+          <t>天赋·体质</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>LP_LegendSeed</t>
+          <t>LP_GiftedScore(3)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -5831,7 +6476,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}注定要成为传奇——只是还没到时候。\n\n- 成为传奇冒险者时一次性获得 10 个传奇属性点\n- 500 / 1000 人形击杀里程碑的传奇属性点奖励翻倍（各 6 点）</t>
+          <t>{PAWN_nameDef}天生结实。\n\n- 体质算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5843,12 +6488,12 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>图腾之魂·熊</t>
+          <t>天赋·智力</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>LP_TotemSpirit(1)</t>
+          <t>LP_GiftedScore(4)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -5858,7 +6503,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>熊的灵魂在{PAWN_nameDef}的血里低吼。\n\n- 总体健康低于 50% 时，受到的非心灵伤害 -35%\n- 疼痛休克阈值 +10%</t>
+          <t>{PAWN_nameDef}天生聪明。\n\n- 智力算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5870,12 +6515,12 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>图腾之魂·狼</t>
+          <t>天赋·感知</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>LP_TotemSpirit(2)</t>
+          <t>LP_GiftedScore(5)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -5885,7 +6530,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>狼群的灵魂跟着{PAWN_nameDef}一起狩猎。\n\n- {PAWN_pronoun}近战命中过的目标（8 秒内），其他友军对它近战命中 +15%\n- 近战命中 10% 让目标倒地 1 秒（体型 3 以上无效）\n- 移动速度 +0</t>
+          <t>{PAWN_nameDef}天生敏锐。\n\n- 感知算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5897,12 +6542,12 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>图腾之魂·鹰</t>
+          <t>天赋·魅力</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>LP_TotemSpirit(3)</t>
+          <t>LP_GiftedScore(6)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -5912,7 +6557,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>鹰的灵魂替{PAWN_nameDef}盯着远处。\n\n- 射击时目标掩体的减免减半（和神射手不叠加）\n- 远程武器射程 ×1.15</t>
+          <t>{PAWN_nameDef}天生讨人喜欢。\n\n- 魅力算作“擅长”：每点正调整值收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5924,12 +6569,12 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>宿敌猎人·龙</t>
+          <t>金刚之躯</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>LP_FavoredEnemy(1)</t>
+          <t>LP_Hardened</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -5939,7 +6584,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}发誓要猎杀世上的龙。\n\n- 对宿敌（龙：五色真龙、力能龙裔、其他龙类）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫宿敌</t>
+          <t>{PAWN_nameDef}的身子骨像铁打的。\n\n- 传奇属性“血量”“承受”“回复”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5951,12 +6596,12 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>宿敌猎人·巨人</t>
+          <t>锋芒</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>LP_FavoredEnemy(2)</t>
+          <t>LP_Edge</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -5966,7 +6611,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}发誓要猎杀巨人。\n\n- 对宿敌（体型 2 以上的巨人种族）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫宿敌施加的眩晕与</t>
+          <t>{PAWN_nameDef}生来就是打仗的料。\n\n- 传奇属性“近战”“远程”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
         </is>
       </c>
     </row>
@@ -5978,12 +6623,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>宿敌猎人·不死</t>
+          <t>灵光</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>LP_FavoredEnemy(3)</t>
+          <t>LP_Insight</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -5993,7 +6638,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}发誓要让死者安息。\n\n- 对宿敌（巫妖、死灵造物、死亡骑士、半巫妖、Anomaly 尸鬼）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害</t>
+          <t>{PAWN_nameDef}的脑子里时常闪过别人想不到的东西。\n\n- 传奇属性“心灵”“学习”每点收益 ×1.5（与种族亲和取较大，不相乘）\n- 智力、感知中较高的一项上限 +2</t>
         </is>
       </c>
     </row>
@@ -6005,12 +6650,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>宿敌猎人·邪魔</t>
+          <t>传奇之胚</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>LP_FavoredEnemy(4)</t>
+          <t>LP_LegendSeed</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -6020,7 +6665,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{PAWN_nameDef}发誓要把邪魔赶回深渊和九狱。\n\n- 对宿敌（深渊恶魔、九狱魔鬼、炎魔、寒冰魔、契约恶魔）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 </t>
+          <t>{PAWN_nameDef}注定要成为传奇——只是还没到时候。\n\n- 成为传奇冒险者时一次性获得 10 个传奇属性点\n- 500 / 1000 人形击杀里程碑的传奇属性点奖励翻倍（各 6 点）</t>
         </is>
       </c>
     </row>
@@ -6032,12 +6677,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>宿敌猎人·异怪</t>
+          <t>图腾之魂·熊</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>LP_FavoredEnemy(5)</t>
+          <t>LP_TotemSpirit(1)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -6047,7 +6692,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}见过幽暗地域里的东西，从此只想把它们杀干净。\n\n- 对宿敌（夺心魔、眼魔、贝希尔、六臂蛇人）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤</t>
+          <t>熊的灵魂在{PAWN_nameDef}的血里低吼。\n\n- 总体健康低于 50% 时，受到的非心灵伤害 -35%\n- 疼痛休克阈值 +10%</t>
         </is>
       </c>
     </row>
@@ -6059,12 +6704,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>宿敌猎人·野兽</t>
+          <t>图腾之魂·狼</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>LP_FavoredEnemy(6)</t>
+          <t>LP_TotemSpirit(2)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -6074,7 +6719,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}是荒野里长大的猎手。\n\n- 对宿敌（动物）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫宿敌施加的眩晕与控制</t>
+          <t>狼群的灵魂跟着{PAWN_nameDef}一起狩猎。\n\n- {PAWN_pronoun}近战命中过的目标（8 秒内），其他友军对它近战命中 +15%\n- 近战命中 10% 让目标倒地 1 秒（体型 3 以上无效）\n- 移动速度 +0</t>
         </is>
       </c>
     </row>
@@ -6086,12 +6731,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>宿敌猎人·仇敌派系</t>
+          <t>图腾之魂·鹰</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>LP_FavoredEnemy(7)</t>
+          <t>LP_TotemSpirit(3)</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -6101,7 +6746,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}和一个派系有血仇（派系名见悬停说明下方）。\n\n- 对宿敌（那个派系的成员）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫</t>
+          <t>鹰的灵魂替{PAWN_nameDef}盯着远处。\n\n- 射击时目标掩体的减免减半（和神射手不叠加）\n- 远程武器射程 ×1.15</t>
         </is>
       </c>
     </row>
@@ -6113,12 +6758,12 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>同调者</t>
+          <t>宿敌猎人·龙</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>LP_Attuner</t>
+          <t>LP_FavoredEnemy(1)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -6128,7 +6773,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>魔法物品在{PAWN_nameDef}手里格外听话。\n\n- 身上魔法物品（1.45.0 魔法物品、魔法衣甲）自带的属性加成 ×1.25\n- 戒指最多戴三枚（平时两枚）\n- {PAWN_pronoun}击杀宿敌冠军时，20% 多掉一件</t>
+          <t>{PAWN_nameDef}发誓要猎杀世上的龙。\n\n- 对宿敌（龙：五色真龙、力能龙裔、其他龙类）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫宿敌</t>
         </is>
       </c>
     </row>
@@ -6140,12 +6785,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>元素之触·火</t>
+          <t>宿敌猎人·巨人</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>LP_ElementTouched(1)</t>
+          <t>LP_FavoredEnemy(2)</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -6155,7 +6800,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>火元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点灼烧伤害\n- 受到的火焰类伤害 -50%\n- {PAWN_possessive}火焰类法术、神术、法杖伤害 +30%\n- 火元素裔：改为火焰伤</t>
+          <t>{PAWN_nameDef}发誓要猎杀巨人。\n\n- 对宿敌（体型 2 以上的巨人种族）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫宿敌施加的眩晕与</t>
         </is>
       </c>
     </row>
@@ -6167,12 +6812,12 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>元素之触·冰</t>
+          <t>宿敌猎人·不死</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>LP_ElementTouched(2)</t>
+          <t>LP_FavoredEnemy(3)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -6182,7 +6827,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>寒冰元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点寒霜伤害，并让目标减速 2 秒\n- 受到的寒冷类伤害 -50%\n- {PAWN_possessive}寒冷类法术、神术、法杖伤害 +30%\n</t>
+          <t>{PAWN_nameDef}发誓要让死者安息。\n\n- 对宿敌（巫妖、死灵造物、死亡骑士、半巫妖、Anomaly 尸鬼）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害</t>
         </is>
       </c>
     </row>
@@ -6194,12 +6839,12 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>元素之触·雷</t>
+          <t>宿敌猎人·邪魔</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>LP_ElementTouched(3)</t>
+          <t>LP_FavoredEnemy(4)</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -6209,7 +6854,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">雷电元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点电击伤害，10% 跳到 2 格内另一个敌人\n- 受到的雷电类伤害 -50%\n- {PAWN_possessive}雷电类法术、神术、法杖伤害 </t>
+          <t xml:space="preserve">{PAWN_nameDef}发誓要把邪魔赶回深渊和九狱。\n\n- 对宿敌（深渊恶魔、九狱魔鬼、炎魔、寒冰魔、契约恶魔）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 </t>
         </is>
       </c>
     </row>
@@ -6221,12 +6866,12 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>元素之触·酸</t>
+          <t>宿敌猎人·异怪</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>LP_ElementTouched(4)</t>
+          <t>LP_FavoredEnemy(5)</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -6236,7 +6881,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>强酸元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点强酸伤害\n- 受到的强酸类伤害 -50%\n- {PAWN_possessive}强酸类法术、神术、法杖伤害 +30%\n- 土元素裔：改为强酸</t>
+          <t>{PAWN_nameDef}见过幽暗地域里的东西，从此只想把它们杀干净。\n\n- 对宿敌（夺心魔、眼魔、贝希尔、六臂蛇人）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤</t>
         </is>
       </c>
     </row>
@@ -6248,12 +6893,12 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>法术抗体</t>
+          <t>宿敌猎人·野兽</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>LP_SpellWarded</t>
+          <t>LP_FavoredEnemy(6)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -6263,7 +6908,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>魔法在{PAWN_nameDef}身上总是打滑。\n\n- 敌方的灵能、法术、神术伤害 -35%（没有武器的伤害、法杖伤害）\n- 敌方的眩晕、魅惑、支配、心灵震爆 50% 无效\n- 只抵抗敌对施法者，友方的增益法术照常生效\n- 代价：</t>
+          <t>{PAWN_nameDef}是荒野里长大的猎手。\n\n- 对宿敌（动物）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫宿敌施加的眩晕与控制</t>
         </is>
       </c>
     </row>
@@ -6275,562 +6920,562 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
+          <t>宿敌猎人·仇敌派系</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>LP_FavoredEnemy(7)</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}和一个派系有血仇（派系名见悬停说明下方）。\n\n- 对宿敌（那个派系的成员）伤害 +25%、命中 +15%\n- 宿敌出现在本地图时提示一次\n- 击杀宿敌累计 50 个后成为“宿敌克星”：伤害 +40%，免疫</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>同调者</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>LP_Attuner</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>魔法物品在{PAWN_nameDef}手里格外听话。\n\n- 身上魔法物品（1.45.0 魔法物品、魔法衣甲）自带的属性加成 ×1.25\n- 戒指最多戴三枚（平时两枚）\n- {PAWN_pronoun}击杀宿敌冠军时，20% 多掉一件</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>元素之触·火</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>LP_ElementTouched(1)</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>火元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点灼烧伤害\n- 受到的火焰类伤害 -50%\n- {PAWN_possessive}火焰类法术、神术、法杖伤害 +30%\n- 火元素裔：改为火焰伤</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>元素之触·冰</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>LP_ElementTouched(2)</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>寒冰元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点寒霜伤害，并让目标减速 2 秒\n- 受到的寒冷类伤害 -50%\n- {PAWN_possessive}寒冷类法术、神术、法杖伤害 +30%\n</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>元素之触·雷</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>LP_ElementTouched(3)</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">雷电元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点电击伤害，10% 跳到 2 格内另一个敌人\n- 受到的雷电类伤害 -50%\n- {PAWN_possessive}雷电类法术、神术、法杖伤害 </t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>元素之触·酸</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>LP_ElementTouched(4)</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>强酸元素在{PAWN_nameDef}身上留下了印记。\n\n- 任何武器命中额外造成 3 点强酸伤害\n- 受到的强酸类伤害 -50%\n- {PAWN_possessive}强酸类法术、神术、法杖伤害 +30%\n- 土元素裔：改为强酸</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>法术抗体</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>LP_SpellWarded</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>魔法在{PAWN_nameDef}身上总是打滑。\n\n- 敌方的灵能、法术、神术伤害 -35%（没有武器的伤害、法杖伤害）\n- 敌方的眩晕、魅惑、支配、心灵震爆 50% 无效\n- 只抵抗敌对施法者，友方的增益法术照常生效\n- 代价：</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
           <t>决斗者</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>LP_Duelist</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>强力特性</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>{PAWN_nameDef}最擅长一对一。\n\n- 身边（1.5 格内）只有一个敌人时：近战命中 +25%、近战闪避 +25%，闪避成功 50% 立即反击一次\n- 被 3 个以上敌人贴身时近战命中 -10%\n（身边敌人数每 4 秒更新</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="7" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
         <is>
           <t>稀有（事迹）</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B92" s="8" t="inlineStr">
         <is>
           <t>屠龙者</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>LP_DeedDragonslayer</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr">
         <is>
           <t>传说事迹</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>{PAWN_nameDef}参与杀死了一条龙。\n\n- 对龙伤害 +30%\n- 免疫龙威带来的惊惧\n- 龙的吐息（龙身上不带武器的伤害）-30%</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="7" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="7" t="inlineStr">
         <is>
           <t>稀有（事迹）</t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B93" s="8" t="inlineStr">
         <is>
           <t>巨人克星</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>LP_Giantbane</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>传说事迹</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr">
         <is>
           <t>{PAWN_nameDef}用近战放倒过三个巨人。\n\n- 近战打体型 1.5 以上的目标伤害 +30%\n- 传奇属性“血量”每点收益至少 ×1.25</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="7" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
         <is>
           <t>稀有（事迹）</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B94" s="8" t="inlineStr">
         <is>
           <t>巫妖克星</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>LP_Lichbane</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>传说事迹</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E94" s="2" t="inlineStr">
         <is>
           <t>{PAWN_nameDef}击败过影巫王拉洛克，或者亲手毁掉过敌人的命匣。\n\n- 对不死生物伤害 +30%\n- 不会被汲取灵魂\n- 传奇属性“心灵”每点收益至少 ×1.25</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="7" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
         <is>
           <t>稀有（事迹）</t>
         </is>
       </c>
-      <c r="B88" s="8" t="inlineStr">
+      <c r="B95" s="8" t="inlineStr">
         <is>
           <t>绝境英雄</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>LP_LastStand</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D95" s="2" t="inlineStr">
         <is>
           <t>传说事迹</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E95" s="2" t="inlineStr">
         <is>
           <t>那一次袭击里，殖民地只剩{PAWN_nameDef}一个人还站着——{PAWN_pronoun}守住了。\n\n- 疼痛休克阈值 +10%\n- 获得时 +1 次属性提升；25% 当场觉醒英雄之资（已有英雄之资、极致或天命时改为 +3 传奇</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="7" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>巧匠之手</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>LP_Artisan</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的手好像天生就知道该怎么用工具。\n\n- 全局工作速度 +10%\n- 传奇属性“工作”每点收益 ×1.5（与种族亲和取较大，不相乘）</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>疾风之足</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>LP_Fleetfoot</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}跑起来像一阵风。\n\n- 移动速度 +0.4\n- 近战闪避 +10</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>钢铁意志</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>LP_IronWill</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的意志像铁一样硬，什么都压不垮。\n\n- 精神崩溃阈值 -8%\n- 心智抗性 +30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>银舌</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>LP_Silvertongue</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}一开口，石头都能被说动。\n\n- 谈判能力 ×1.3、社交影响 ×1.3\n- 魅力上限 +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>荒野之躯</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>LP_Hardy</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}在荒野里摸爬滚打长大，什么苦都吃过。\n\n- 免疫获得速度 ×1.2\n- 伤口愈合速度 ×1.3\n- 毒素抗性 +25%\n- 舒适温度范围两头各放宽 10°C</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>远瞳</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>LP_EagleEyed</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>强力特性</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}能看清别人只看得到一个黑点的东西。\n\n- 射击精度 +6\n- 瞄准时间 ×0.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="15" t="inlineStr">
+        <is>
+          <t>稀有（诅咒）</t>
+        </is>
+      </c>
+      <c r="B102" s="16" t="inlineStr">
+        <is>
+          <t>厄运缠身</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>LP_Doomed</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>一个女巫在临死前诅咒了{PAWN_nameDef}。厄运一直跟着{PAWN_objective}，有时也会扑向别人。\n\n- 近战闪避 +15\n- 被敌人打中时 15% 的几率「厄运转嫁」：攻击者也受到这次伤害的一半\n- 代价：平均每</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="15" t="inlineStr">
+        <is>
+          <t>稀有（诅咒）</t>
+        </is>
+      </c>
+      <c r="B103" s="16" t="inlineStr">
+        <is>
+          <t>空心之人</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>LP_Hollow</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的一半灵魂被什么东西吃掉了，剩下的那一半很平静——平静得吓人。\n\n- 精神崩溃阈值 -15%\n- 疼痛休克阈值 +20%\n- 心智抗性 +50%\n- 代价：社交影响 ×0.5、技能学习速度 ×0.8、心</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="7" t="inlineStr">
         <is>
           <t>优秀（事迹）</t>
         </is>
       </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="B104" s="8" t="inlineStr">
         <is>
           <t>圣徒</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>LP_Saint</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
         <is>
           <t>传说事迹</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr">
         <is>
           <t>[PAWN_nameDef]在异端勇者面前证了道，是[PAWN_possessive]神的圣徒：心灵敏感度+15%、社交+2；[PAWN_possessive]的神每天神眷+0.2。装了 VPE 时神恩强度+0.15。</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B90" s="4" t="inlineStr">
-        <is>
-          <t>屠龙志士</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>LP_DragonStance(1)</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}发过誓，这辈子要亲手斩下一条龙。\n\n- 对龙的伤害 +20%（和其他类型伤害加成合计最多 +60%）\n- 击杀龙：心情 +10，持续 10 天\n- 对殖民地的龙裔好感 -10\n- 龙裔不会有这个特性</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B91" s="4" t="inlineStr">
-        <is>
-          <t>巨人杀手</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>LP_GiantStance(-1)</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}专门学过怎么对付比自己高三倍的东西。\n\n- 近战攻击体型 1.5 以上的目标伤害 +20%（和其他类型伤害加成合计最多 +60%）\n- 躲闪体型 1.5 以上敌人的近战攻击 +10%\n- 对巨人好感 -1</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>不死猎人</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>LP_UndeadStance(-1)</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}把一辈子都花在了让死者安息上。\n\n- 对不死生物的伤害 +20%（和其他类型伤害加成合计最多 +60%）\n- 殖民地有巫妖或死灵造物：心情 -6\n- 巫妖和不死种族不会有这个特性</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>殖巢幸存者</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>LP_HiveSurvivor</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}从夺心魔的殖巢里活着逃了出来。\n\n- 心智抗性 +50%\n- 地图上有夺心魔：心情 -4\n- 对吉斯洋基好感 +10\n- “逃离殖巢”开局的人类俘虏必带\n- 夺心魔和半夺心魔不会有这个特性</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B94" s="4" t="inlineStr">
-        <is>
-          <t>战术家</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>LP_Tactician</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}天生会看战场。\n\n- 被征召时，4 格内的友军近战与射击命中 +5%（多个战术家不叠加）\n- 装了 VPE 时：战士路径经验 +25%（和背景、魔网之子等的经验加成取较高，不叠加）</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>奥术天赋</t>
-        </is>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>LP_ArcaneGift</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}对魔网的流动格外敏感。\n\n- 装了 VPE 时：法师路径经验 +25%（与其他经验加成取较高），心灵熵消耗 -10%\n- 没装 VPE 时：心灵敏感度 +10%\n- 不会和狂野魔法同时出现</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B96" s="4" t="inlineStr">
-        <is>
-          <t>狂野魔法</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>LP_WildMagic</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}身上的魔力从来不太听话。\n\n- 装了 VPE 时：每次施放能力有 5% 的几率引发魔力浪涌；法术伤害 +10%\n- 没装 VPE 时：每天随机一次小浪涌\n- 浪涌共 12 种：隐身 10 秒、脚下长花、敌</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>机械迷</t>
-        </is>
-      </c>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t>LP_Tinkerer</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}看见齿轮就挪不开眼。\n\n- 修理建筑速度 +20%\n- 装了 VPE 时：器械师路径经验 +25%（与其他经验加成取较高），火器射击冷却 -5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B98" s="4" t="inlineStr">
-        <is>
-          <t>自然之子</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>LP_NatureBond</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}在林子里比在屋里自在。\n\n- 待在户外：心情 +2\n- 驯服、训练动物的成功率 +15%\n- 装了 VPE 时：德鲁伊路径经验 +25%（与其他经验加成取较高）</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>寻宝狂</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
-        <is>
-          <t>LP_TreasureHunter</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}听到“宝藏”两个字就坐不住。\n\n- 法师塔坠落、进入迷锁地牢：心情 +5「冒险的召唤」\n- 拆除古代遗迹多得 20% 材料\n- 有寻宝狂在迷锁地牢里时，地牢的宝物有 10% 的几率多出一件</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B100" s="4" t="inlineStr">
-        <is>
-          <t>安息之魂</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>LP_Revenant(1)</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>诅咒之力</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}的血仇已经报了，亡魂终于安息。\n\n- 对昔日凶手所在派系的伤害 +15%（和其他类型伤害加成合计最多 +60%）\n- 不再死后复活</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="7" t="inlineStr">
-        <is>
-          <t>优秀（事迹）</t>
-        </is>
-      </c>
-      <c r="B101" s="8" t="inlineStr">
-        <is>
-          <t>冥界归来</t>
-        </is>
-      </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>LP_DeathReturned</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>传说事迹</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}死过一次，又回来了。\n\n- 不会因为死亡类事件（亲友、同伴死去，目睹死亡）心情变差\n- 对不死生物伤害 +20%\n- 每 30 天一次：倒地后 2 小时内不会失血而死</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B102" s="4" t="inlineStr">
-        <is>
-          <t>侍僧</t>
-        </is>
-      </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>LP_Background_Acolyte</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>背景特性</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}曾在神殿里侍奉，习惯了祈祷与静修。\n\n- 冥想心灵专注获取 +20%\n- 参加任何意识形态仪式后获得心情 +3“神圣时光”（1天）\n- 装了 Vanilla Psycasts Expanded 时：牧师路</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>罪犯</t>
-        </is>
-      </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>LP_Background_Criminal</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>背景特性</t>
-        </is>
-      </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{PAWN_nameDef}在城市的阴影里讨过生活，撬锁、销赃、躲卫兵都是老本行。\n\n- 作为囚犯时越狱几率 ×2\n- 殖民地有罪犯背景的殖民者时，囚犯越狱几率 ×0.75（{PAWN_pronoun}知道犯人会从哪里钻空子）\n- </t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="3" t="inlineStr">
-        <is>
-          <t>优秀</t>
-        </is>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>民间英雄</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>LP_Background_FolkHero</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>背景特性</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}曾经挺身对抗暴君和怪物，乡亲们至今还在传唱{PAWN_possessive}故事。\n\n- 被征召时，6格内的其他殖民者心情 +3“英雄在此”\n- {PAWN_pronoun}倒地时，全殖民地心情 -3“英雄</t>
         </is>
       </c>
     </row>
@@ -6842,22 +7487,22 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>贵族</t>
+          <t>屠龙志士</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>LP_Background_Noble</t>
+          <t>LP_DragonStance(1)</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>背景特性</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}出身名门，从小就被教导如何发号施令，而不是如何拿扫帚。\n\n- 社交影响 +15%\n- 不做清洁和搬运\n- 卧室印象低于“体面”时心情 -4“配不上我的身份”\n- 装了皇权 DLC 时：获得荣誉 ×1.2</t>
+          <t>{PAWN_nameDef}发过誓，这辈子要亲手斩下一条龙。\n\n- 对龙的伤害 +20%（和其他类型伤害加成合计最多 +60%）\n- 击杀龙：心情 +10，持续 10 天\n- 对殖民地的龙裔好感 -10\n- 龙裔不会有这个特性</t>
         </is>
       </c>
     </row>
@@ -6869,22 +7514,22 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>贤者</t>
+          <t>巨人杀手</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>LP_Background_Sage</t>
+          <t>LP_GiantStance(-1)</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>背景特性</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}在图书馆和学院里度过了大半生，离开书本就浑身不自在。\n\n- 研究速度 +10%\n- 读书收益 +30%\n- 装了 Vanilla Psycasts Expanded 时：法师路径经验 +25%\n- 殖民</t>
+          <t>{PAWN_nameDef}专门学过怎么对付比自己高三倍的东西。\n\n- 近战攻击体型 1.5 以上的目标伤害 +20%（和其他类型伤害加成合计最多 +60%）\n- 躲闪体型 1.5 以上敌人的近战攻击 +10%\n- 对巨人好感 -1</t>
         </is>
       </c>
     </row>
@@ -6896,22 +7541,22 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>士兵</t>
+          <t>不死猎人</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>LP_Background_Soldier</t>
+          <t>LP_UndeadStance(-1)</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>背景特性</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}在军队里服过役，听到号令身体就会自己动起来。\n\n- 被征召时瞄准时间 -10%\n- 3格内有另一名士兵背景的友军时，双方射击精度和近战命中 +5%</t>
+          <t>{PAWN_nameDef}把一辈子都花在了让死者安息上。\n\n- 对不死生物的伤害 +20%（和其他类型伤害加成合计最多 +60%）\n- 殖民地有巫妖或死灵造物：心情 -6\n- 巫妖和不死种族不会有这个特性</t>
         </is>
       </c>
     </row>
@@ -6923,22 +7568,22 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>隐士</t>
+          <t>殖巢幸存者</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>LP_Background_Hermit</t>
+          <t>LP_HiveSurvivor</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>背景特性</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>{PAWN_nameDef}曾经独自在荒野里隐居多年，比起人群更习惯和自己的念头相处。\n\n- 独占卧室时心情 +3“独处之所”\n- 和别人同住一间卧室时心情 -4“没有清静”（替代原版的“睡在营房”心情）\n- 冥想心灵专注获取 +3</t>
+          <t>{PAWN_nameDef}从夺心魔的殖巢里活着逃了出来。\n\n- 心智抗性 +50%\n- 地图上有夺心魔：心情 -4\n- 对吉斯洋基好感 +10\n- “逃离殖巢”开局的人类俘虏必带\n- 夺心魔和半夺心魔不会有这个特性</t>
         </is>
       </c>
     </row>
@@ -6950,427 +7595,427 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
+          <t>战术家</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>LP_Tactician</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}天生会看战场。\n\n- 被征召时，4 格内的友军近战与射击命中 +5%（多个战术家不叠加）\n- 装了 VPE 时：战士路径经验 +25%（和背景、魔网之子等的经验加成取较高，不叠加）</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>奥术天赋</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>LP_ArcaneGift</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}对魔网的流动格外敏感。\n\n- 装了 VPE 时：法师路径经验 +25%（与其他经验加成取较高），心灵熵消耗 -10%\n- 没装 VPE 时：心灵敏感度 +10%\n- 不会和狂野魔法同时出现</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>狂野魔法</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>LP_WildMagic</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}身上的魔力从来不太听话。\n\n- 装了 VPE 时：每次施放能力有 5% 的几率引发魔力浪涌；法术伤害 +10%\n- 没装 VPE 时：每天随机一次小浪涌\n- 浪涌共 12 种：隐身 10 秒、脚下长花、敌</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>机械迷</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>LP_Tinkerer</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}看见齿轮就挪不开眼。\n\n- 修理建筑速度 +20%\n- 装了 VPE 时：器械师路径经验 +25%（与其他经验加成取较高），火器射击冷却 -5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>自然之子</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>LP_NatureBond</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}在林子里比在屋里自在。\n\n- 待在户外：心情 +2\n- 驯服、训练动物的成功率 +15%\n- 装了 VPE 时：德鲁伊路径经验 +25%（与其他经验加成取较高）</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>寻宝狂</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>LP_TreasureHunter</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}听到“宝藏”两个字就坐不住。\n\n- 法师塔坠落、进入迷锁地牢：心情 +5「冒险的召唤」\n- 拆除古代遗迹多得 20% 材料\n- 有寻宝狂在迷锁地牢里时，地牢的宝物有 10% 的几率多出一件</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>安息之魂</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>LP_Revenant(1)</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>诅咒之力</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}的血仇已经报了，亡魂终于安息。\n\n- 对昔日凶手所在派系的伤害 +15%（和其他类型伤害加成合计最多 +60%）\n- 不再死后复活</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>优秀（事迹）</t>
+        </is>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>冥界归来</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>LP_DeathReturned</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>传说事迹</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}死过一次，又回来了。\n\n- 不会因为死亡类事件（亲友、同伴死去，目睹死亡）心情变差\n- 对不死生物伤害 +20%\n- 每 30 天一次：倒地后 2 小时内不会失血而死</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>侍僧</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>LP_Background_Acolyte</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>背景特性</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}曾在神殿里侍奉，习惯了祈祷与静修。\n\n- 冥想心灵专注获取 +20%\n- 参加任何意识形态仪式后获得心情 +3“神圣时光”（1天）\n- 装了 Vanilla Psycasts Expanded 时：牧师路</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>罪犯</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>LP_Background_Criminal</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>背景特性</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{PAWN_nameDef}在城市的阴影里讨过生活，撬锁、销赃、躲卫兵都是老本行。\n\n- 作为囚犯时越狱几率 ×2\n- 殖民地有罪犯背景的殖民者时，囚犯越狱几率 ×0.75（{PAWN_pronoun}知道犯人会从哪里钻空子）\n- </t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>民间英雄</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>LP_Background_FolkHero</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>背景特性</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}曾经挺身对抗暴君和怪物，乡亲们至今还在传唱{PAWN_possessive}故事。\n\n- 被征召时，6格内的其他殖民者心情 +3“英雄在此”\n- {PAWN_pronoun}倒地时，全殖民地心情 -3“英雄</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>贵族</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>LP_Background_Noble</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>背景特性</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}出身名门，从小就被教导如何发号施令，而不是如何拿扫帚。\n\n- 社交影响 +15%\n- 不做清洁和搬运\n- 卧室印象低于“体面”时心情 -4“配不上我的身份”\n- 装了皇权 DLC 时：获得荣誉 ×1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>贤者</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>LP_Background_Sage</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>背景特性</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}在图书馆和学院里度过了大半生，离开书本就浑身不自在。\n\n- 研究速度 +10%\n- 读书收益 +30%\n- 装了 Vanilla Psycasts Expanded 时：法师路径经验 +25%\n- 殖民</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>士兵</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>LP_Background_Soldier</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>背景特性</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}在军队里服过役，听到号令身体就会自己动起来。\n\n- 被征召时瞄准时间 -10%\n- 3格内有另一名士兵背景的友军时，双方射击精度和近战命中 +5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>隐士</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>LP_Background_Hermit</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>背景特性</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}曾经独自在荒野里隐居多年，比起人群更习惯和自己的念头相处。\n\n- 独占卧室时心情 +3“独处之所”\n- 和别人同住一间卧室时心情 -4“没有清静”（替代原版的“睡在营房”心情）\n- 冥想心灵专注获取 +3</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>优秀</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
           <t>局外人</t>
         </is>
       </c>
-      <c r="C109" s="2" t="inlineStr">
+      <c r="C124" s="2" t="inlineStr">
         <is>
           <t>LP_Background_Outlander</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
+      <c r="D124" s="2" t="inlineStr">
         <is>
           <t>背景特性</t>
         </is>
       </c>
-      <c r="E109" s="2" t="inlineStr">
+      <c r="E124" s="2" t="inlineStr">
         <is>
           <t>{PAWN_nameDef}在文明之外的荒原上长大，风雨对{PAWN_objective}来说就是日常。\n\n- 在没有屋顶、也不在居住区的地方移动速度 +10%\n- 采集野生植物产量 +25%\n- 不受淋湿、沙尘等坏天气心情影响\n</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>守序</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>LP_Order(1)</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}相信规矩、秩序和说到做到。\n\n- 作息表“工作”时段内全局工作速度 +5%\n- 不会发生纵火、乱跑、出走类精神崩溃\n- 殖民地有领袖或头衔持有者：心情 +3「秩序井然」\n- 自己的作息表全是“任意”：心</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>混乱</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>LP_Order(-1)</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}讨厌被管着，想到什么就做什么。\n\n- 灵感出现的几率 ×1.5\n- 连续征召超过 6 小时：心情 -4「被管束」</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>仁善</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>LP_Morality(1)</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}心地善良，见不得别人受苦。\n\n- 救援倒地的人、给囚犯包扎：心情 +2「善举」\n- 用制伏武器打倒敌人（不伤性命）：心情 +2「手下留情」\n- 处决、摘取器官带来的坏心情之外再 -5「良心不安」\n- 殖</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B113" s="2" t="inlineStr">
-        <is>
-          <t>邪恶</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>LP_Morality(-1)</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E113" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}只在乎自己想要什么，别人的痛苦不算什么。\n\n- 处决、摘取器官、奴役不会让{PAWN_objective}心情变差\n- 压制奴隶的效果 +20%\n- 殖民地有巫妖：心情 +2「黑暗庇护」\n- 不会和善良</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>惧龙</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>LP_DragonStance(-1)</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}小时候见过龙烧掉一整座村子。\n\n- 地图上有龙：心情 -6「龙威压顶」\n- 龙在 10 格内时，每隔几秒有 10% 的几率掉头逃开\n- 龙裔和五色真龙不会有这个特性</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr">
-        <is>
-          <t>巨人仆从</t>
-        </is>
-      </c>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>LP_GiantStance(1)</t>
-        </is>
-      </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}在巨人的宅邸里长大，跟在大个子身边才踏实。\n\n- 在体型 1.5 以上的殖民者 3 格内干活，全局工作速度 +10%\n- 对体型 1.5 以上的殖民者好感 +15</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>巫妖信徒</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>LP_UndeadStance(1)</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}相信不朽的巫妖才是这个世界真正的主人。\n\n- 殖民地有巫妖：心情 +4</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B117" s="2" t="inlineStr">
-        <is>
-          <t>世界公民</t>
-        </is>
-      </c>
-      <c r="C117" s="2" t="inlineStr">
-        <is>
-          <t>LP_RaceAttitude(1)</t>
-        </is>
-      </c>
-      <c r="D117" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E117" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}走过很多地方，和哪个种族都处得来。\n\n- 不受种族关系的负面心情影响\n- 殖民地每多一个种族，心情 +1（最多 +4）</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="inlineStr">
-        <is>
-          <t>纯血至上</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>LP_RaceAttitude(-1)</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}觉得只有自己的种族靠得住。\n\n- 对同种族的人好感 +10，对其他种族 -10\n- 本种族在殖民地占多数：心情 +3，否则 -3</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="inlineStr">
-        <is>
-          <t>龙之眷从</t>
-        </is>
-      </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>LP_DragonServant</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}的祖辈世代侍奉龙。\n\n- 殖民地有龙裔殖民者：心情 +4\n- 把东西搬进龙裔的宝库时移动速度 +30%\n- 不会从龙宝库里往外搬东西\n- 殖民地的龙死去：心情 -15\n- 狗头人出现这个特性的几率 ×</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B120" s="2" t="inlineStr">
-        <is>
-          <t>吉斯流亡者</t>
-        </is>
-      </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>LP_GithExile</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E120" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}背弃了巫妖女王维拉基斯。\n\n- 不再因为见到殖民地的巫妖而高兴（替代吉斯洋基原有的巫妖心情）\n- 对巫妖好感 -10\n- 只会出现在吉斯洋基身上</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>魔法恐惧</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>LP_Magephobe</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}不信任任何会施法的人。\n\n- 对有灵能、会施法的人好感 -10\n- 被别人施加增益法术：心情 -3\n- 受到敌方法术的伤害 -10%</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>秘法上瘾</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>LP_ArcaneCraving</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E122" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}迷上了魔法流过身体的感觉。\n\n- 超过 5 天没用过魔法药水或魔法卷轴：心情 -6「秘法渴求」\n- 用了一瓶魔法药水或一张魔法卷轴：心情 +4，持续 2 天</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B123" s="2" t="inlineStr">
-        <is>
-          <t>位面错乱</t>
-        </is>
-      </c>
-      <c r="C123" s="2" t="inlineStr">
-        <is>
-          <t>LP_PlaneTouched</t>
-        </is>
-      </c>
-      <c r="D123" s="2" t="inlineStr">
-        <is>
-          <t>性格特性</t>
-        </is>
-      </c>
-      <c r="E123" s="2" t="inlineStr">
-        <is>
-          <t>{PAWN_nameDef}曾在两个位面之间迷失了很久。\n\n- 位面裂隙里钻出来的野兽不会主动攻击{PAWN_objective}\n- 每 10～15 天会出神 1 小时\n- 传送类能力冷却 -20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>普通</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t>信徒（洛山达）</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>LP_Devotee(1)</t>
-        </is>
-      </c>
-      <c r="D124" s="2" t="inlineStr">
-        <is>
-          <t>信仰</t>
-        </is>
-      </c>
-      <c r="E124" s="2" t="inlineStr">
-        <is>
-          <t>[PAWN_nameDef]是晨曦之神洛山达的信徒：在圣坛祈祷得到的神眷翻倍；种植速度+10%。殖民地的守护神是洛山达时心情+4，是他的敌对神时心情-6。</t>
         </is>
       </c>
     </row>
@@ -7382,22 +8027,22 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>信徒（提尔）</t>
+          <t>守序</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(2)</t>
+          <t>LP_Order(1)</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是正义之神提尔的信徒：在圣坛祈祷得到的神眷翻倍；和人打架的可能-25%。殖民地的守护神是提尔时心情+4，是他的敌对神时心情-6。</t>
+          <t>{PAWN_nameDef}相信规矩、秩序和说到做到。\n\n- 作息表“工作”时段内全局工作速度 +5%\n- 不会发生纵火、乱跑、出走类精神崩溃\n- 殖民地有领袖或头衔持有者：心情 +3「秩序井然」\n- 自己的作息表全是“任意”：心</t>
         </is>
       </c>
     </row>
@@ -7409,22 +8054,22 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>信徒（密斯特拉）</t>
+          <t>混乱</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(3)</t>
+          <t>LP_Order(-1)</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是魔法女神密斯特拉的信徒：在圣坛祈祷得到的神眷翻倍；心灵敏感度+10%。殖民地的守护神是密斯特拉时心情+4，是她的敌对神时心情-6。</t>
+          <t>{PAWN_nameDef}讨厌被管着，想到什么就做什么。\n\n- 灵感出现的几率 ×1.5\n- 连续征召超过 6 小时：心情 -4「被管束」</t>
         </is>
       </c>
     </row>
@@ -7436,22 +8081,22 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>信徒（凯兰沃）</t>
+          <t>仁善</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(4)</t>
+          <t>LP_Morality(1)</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是死亡之神凯兰沃的信徒：在圣坛祈祷得到的神眷翻倍；手术成功率+5%，看到尸体不难受。殖民地的守护神是凯兰沃时心情+4。</t>
+          <t>{PAWN_nameDef}心地善良，见不得别人受苦。\n\n- 救援倒地的人、给囚犯包扎：心情 +2「善举」\n- 用制伏武器打倒敌人（不伤性命）：心情 +2「手下留情」\n- 处决、摘取器官带来的坏心情之外再 -5「良心不安」\n- 殖</t>
         </is>
       </c>
     </row>
@@ -7463,22 +8108,22 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>信徒（马拉尔）</t>
+          <t>邪恶</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(5)</t>
+          <t>LP_Morality(-1)</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是狩猎之神马拉尔的信徒：在圣坛祈祷得到的神眷翻倍；打猎时命中+10%。殖民地的守护神是马拉尔时心情+4，是他的敌对神时心情-6。</t>
+          <t>{PAWN_nameDef}只在乎自己想要什么，别人的痛苦不算什么。\n\n- 处决、摘取器官、奴役不会让{PAWN_objective}心情变差\n- 压制奴隶的效果 +20%\n- 殖民地有巫妖：心情 +2「黑暗庇护」\n- 不会和善良</t>
         </is>
       </c>
     </row>
@@ -7490,22 +8135,22 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>信徒（塔洛斯）</t>
+          <t>惧龙</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(6)</t>
+          <t>LP_DragonStance(-1)</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是风暴之神塔洛斯的信徒：在圣坛祈祷得到的神眷翻倍；雷暴天心情+3。殖民地的守护神是塔洛斯时心情+4，是他的敌对神时心情-6。</t>
+          <t>{PAWN_nameDef}小时候见过龙烧掉一整座村子。\n\n- 地图上有龙：心情 -6「龙威压顶」\n- 龙在 10 格内时，每隔几秒有 10% 的几率掉头逃开\n- 龙裔和五色真龙不会有这个特性</t>
         </is>
       </c>
     </row>
@@ -7517,22 +8162,22 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>信徒（班恩）</t>
+          <t>巨人仆从</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(7)</t>
+          <t>LP_GiantStance(1)</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是暴政之神班恩的信徒：在圣坛祈祷得到的神眷翻倍；镇压奴隶的效果+20%。殖民地的守护神是班恩时心情+4，是他的敌对神时心情-6。</t>
+          <t>{PAWN_nameDef}在巨人的宅邸里长大，跟在大个子身边才踏实。\n\n- 在体型 1.5 以上的殖民者 3 格内干活，全局工作速度 +10%\n- 对体型 1.5 以上的殖民者好感 +15</t>
         </is>
       </c>
     </row>
@@ -7544,22 +8189,22 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>信徒（莎尔）</t>
+          <t>巫妖信徒</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(8)</t>
+          <t>LP_UndeadStance(1)</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是黑暗之神莎尔的信徒：在圣坛祈祷得到的神眷翻倍；在黑暗里不会难受。殖民地的守护神是莎尔时心情+4，是她的敌对神时心情-6。</t>
+          <t>{PAWN_nameDef}相信不朽的巫妖才是这个世界真正的主人。\n\n- 殖民地有巫妖：心情 +4</t>
         </is>
       </c>
     </row>
@@ -7571,22 +8216,22 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>信徒（苏尔特）</t>
+          <t>世界公民</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(9)</t>
+          <t>LP_RaceAttitude(1)</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]是火巨人之王苏尔特的信徒：在圣坛祈祷得到的神眷翻倍；锻造速度+10%。殖民地的守护神是苏尔特时心情+4。</t>
+          <t>{PAWN_nameDef}走过很多地方，和哪个种族都处得来。\n\n- 不受种族关系的负面心情影响\n- 殖民地每多一个种族，心情 +1（最多 +4）</t>
         </is>
       </c>
     </row>
@@ -7598,22 +8243,22 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>信徒（伊尔斯维）</t>
+          <t>纯血至上</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(10)</t>
+          <t>LP_RaceAttitude(-1)</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]侍奉夺心魔之神伊尔斯维。</t>
+          <t>{PAWN_nameDef}觉得只有自己的种族靠得住。\n\n- 对同种族的人好感 +10，对其他种族 -10\n- 本种族在殖民地占多数：心情 +3，否则 -3</t>
         </is>
       </c>
     </row>
@@ -7625,22 +8270,22 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>信徒（维拉基斯）</t>
+          <t>龙之眷从</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>LP_Devotee(11)</t>
+          <t>LP_DragonServant</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>性格特性</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>[PAWN_nameDef]侍奉巫妖女王维拉基斯。</t>
+          <t>{PAWN_nameDef}的祖辈世代侍奉龙。\n\n- 殖民地有龙裔殖民者：心情 +4\n- 把东西搬进龙裔的宝库时移动速度 +30%\n- 不会从龙宝库里往外搬东西\n- 殖民地的龙死去：心情 -15\n- 狗头人出现这个特性的几率 ×</t>
         </is>
       </c>
     </row>
@@ -7652,27 +8297,432 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
+          <t>吉斯流亡者</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>LP_GithExile</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}背弃了巫妖女王维拉基斯。\n\n- 不再因为见到殖民地的巫妖而高兴（替代吉斯洋基原有的巫妖心情）\n- 对巫妖好感 -10\n- 只会出现在吉斯洋基身上</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>魔法恐惧</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>LP_Magephobe</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}不信任任何会施法的人。\n\n- 对有灵能、会施法的人好感 -10\n- 被别人施加增益法术：心情 -3\n- 受到敌方法术的伤害 -10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>秘法上瘾</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>LP_ArcaneCraving</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}迷上了魔法流过身体的感觉。\n\n- 超过 5 天没用过魔法药水或魔法卷轴：心情 -6「秘法渴求」\n- 用了一瓶魔法药水或一张魔法卷轴：心情 +4，持续 2 天</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>位面错乱</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>LP_PlaneTouched</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>性格特性</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>{PAWN_nameDef}曾在两个位面之间迷失了很久。\n\n- 位面裂隙里钻出来的野兽不会主动攻击{PAWN_objective}\n- 每 10～15 天会出神 1 小时\n- 传送类能力冷却 -20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>信徒（洛山达）</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(1)</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是晨曦之神洛山达的信徒：在圣坛祈祷得到的神眷翻倍；种植速度+10%。殖民地的守护神是洛山达时心情+4，是他的敌对神时心情-6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>信徒（提尔）</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(2)</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是正义之神提尔的信徒：在圣坛祈祷得到的神眷翻倍；和人打架的可能-25%。殖民地的守护神是提尔时心情+4，是他的敌对神时心情-6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>信徒（密斯特拉）</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(3)</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是魔法女神密斯特拉的信徒：在圣坛祈祷得到的神眷翻倍；心灵敏感度+10%。殖民地的守护神是密斯特拉时心情+4，是她的敌对神时心情-6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>信徒（凯兰沃）</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(4)</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是死亡之神凯兰沃的信徒：在圣坛祈祷得到的神眷翻倍；手术成功率+5%，看到尸体不难受。殖民地的守护神是凯兰沃时心情+4。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>信徒（马拉尔）</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(5)</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是狩猎之神马拉尔的信徒：在圣坛祈祷得到的神眷翻倍；打猎时命中+10%。殖民地的守护神是马拉尔时心情+4，是他的敌对神时心情-6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>信徒（塔洛斯）</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(6)</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是风暴之神塔洛斯的信徒：在圣坛祈祷得到的神眷翻倍；雷暴天心情+3。殖民地的守护神是塔洛斯时心情+4，是他的敌对神时心情-6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>信徒（班恩）</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(7)</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是暴政之神班恩的信徒：在圣坛祈祷得到的神眷翻倍；镇压奴隶的效果+20%。殖民地的守护神是班恩时心情+4，是他的敌对神时心情-6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>信徒（莎尔）</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(8)</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是黑暗之神莎尔的信徒：在圣坛祈祷得到的神眷翻倍；在黑暗里不会难受。殖民地的守护神是莎尔时心情+4，是她的敌对神时心情-6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>信徒（苏尔特）</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(9)</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]是火巨人之王苏尔特的信徒：在圣坛祈祷得到的神眷翻倍；锻造速度+10%。殖民地的守护神是苏尔特时心情+4。</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>信徒（伊尔斯维）</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(10)</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]侍奉夺心魔之神伊尔斯维。</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>信徒（维拉基斯）</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>LP_Devotee(11)</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>信仰</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>[PAWN_nameDef]侍奉巫妖女王维拉基斯。</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
           <t>无神者</t>
         </is>
       </c>
-      <c r="C135" s="2" t="inlineStr">
+      <c r="C150" s="2" t="inlineStr">
         <is>
           <t>LP_Atheist</t>
         </is>
       </c>
-      <c r="D135" s="2" t="inlineStr">
+      <c r="D150" s="2" t="inlineStr">
         <is>
           <t>信仰</t>
         </is>
       </c>
-      <c r="E135" s="2" t="inlineStr">
+      <c r="E150" s="2" t="inlineStr">
         <is>
           <t>[PAWN_nameDef]不信任何神：不受信仰相关的心情影响，不会祈祷，戴圣徽也没用；神术落在[PAWN_objective]身上只有一半效果；心智抗性+10%。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E135"/>
+  <autoFilter ref="A1:E150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7683,7 +8733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8938,55 +9988,63 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>天赋·力量/天赋·敏捷/天赋·体质/天赋·智力/天赋·感知/天赋·魅力</t>
+          <t>法术抗体</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>LP_GiftedScore</t>
+          <t>LP_SpellWarded</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Isekai 力大 / 敏捷 / 坚韧 / 聪慧 / 开悟 / 巧舌</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr"/>
+          <t>魔裔之血</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>LP_Spellblood</t>
+        </is>
+      </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>装了 Isekai 时，天赋·某项和对应属性的 Isekai 白色属性特性互斥（代码按等级判断，HeroTraitsIsekai.cs）</t>
+          <t>定义里写明互斥（conflictingTraits）</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>仁善</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr"/>
+          <t>天赋·力量/天赋·敏捷/天赋·体质/天赋·智力/天赋·感知/天赋·魅力</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>LP_GiftedScore</t>
+        </is>
+      </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>原版：心理变态、原版：嗜血、巫妖信徒</t>
+          <t>Isekai 力大 / 敏捷 / 坚韧 / 聪慧 / 开悟 / 巧舌</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>代码互斥（DndTraits.Clash，按等级）</t>
+          <t>装了 Isekai 时，天赋·某项和对应属性的 Isekai 白色属性特性互斥（代码按等级判断，HeroTraitsIsekai.cs）</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>邪恶</t>
+          <t>仁善</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr"/>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>原版：善良、不死猎人</t>
+          <t>原版：心理变态、原版：嗜血、巫妖信徒</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr"/>
@@ -8999,43 +10057,62 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>狂野魔法</t>
+          <t>邪恶</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>奥术天赋、魔法恐惧</t>
+          <t>原版：善良、不死猎人</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>代码互斥（DndTraits.Clash）</t>
+          <t>代码互斥（DndTraits.Clash，按等级）</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>守序/混乱</t>
+          <t>狂野魔法</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr"/>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>仁善/邪恶</t>
+          <t>奥术天赋、魔法恐惧</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
+          <t>代码互斥（DndTraits.Clash）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>守序/混乱</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>仁善/邪恶</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
           <t>阵营类每人最多 1 个（性格特性生成时）</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E51"/>
+  <autoFilter ref="A1:E52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9100,32 +10177,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>稀有天赋之间互斥（每人最多 1 个）</t>
+          <t>诅咒之力之间互斥（每人最多 1 个诅咒）</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>LP_PointTalent</t>
+          <t>LP_Curse</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>凡人之志、大器晚成、天赋异禀、百炼成钢</t>
+          <t>兽化症·狼/兽化症·熊/兽化症·虎、厄运缠身、吸血鬼之咒、复仇亡魂/安息之魂、狱火烙印、空心之人、远域之触</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>天命之间互斥（每人最多 1 个天命）</t>
+          <t>稀有天赋之间互斥（每人最多 1 个）</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>LP_Destiny</t>
+          <t>LP_PointTalent</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -9133,27 +10210,27 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>神之勇士·洛山达/神之勇士·提尔/神之勇士·密斯特拉/神之勇士·凯兰沃/神之勇士·马拉尔/神之勇士·塔洛斯/神之勇士·班恩/神之勇士·莎尔/神之勇士·苏尔特、邪契者·邪魔/邪契者·妖精/邪契者·旧日、预言之子、魔网之子</t>
+          <t>凡人之志、大器晚成、天赋异禀、百炼成钢</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>诅咒之力之间互斥（每人最多 1 个诅咒）</t>
+          <t>天命之间互斥（每人最多 1 个天命）</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>LP_Curse</t>
+          <t>LP_Destiny</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>兽化症·狼/兽化症·熊/兽化症·虎、复仇亡魂/安息之魂、远域之触</t>
+          <t>神之勇士·洛山达/神之勇士·提尔/神之勇士·密斯特拉/神之勇士·凯兰沃/神之勇士·马拉尔/神之勇士·塔洛斯/神之勇士·班恩/神之勇士·莎尔/神之勇士·苏尔特、邪契者·邪魔/邪契者·妖精/邪契者·旧日、预言之子、魔网之子</t>
         </is>
       </c>
     </row>

</xml_diff>